<commit_message>
exclusão tomar do geru da listagem
</commit_message>
<xml_diff>
--- a/nome_clientes.xlsx
+++ b/nome_clientes.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FernandoHenriqueSofi\Desktop\Monitoramento\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FernandoHenriqueSofi\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8C9D28D-9DA3-40DD-9DDB-2FCAC77B74BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADD9A644-77AE-4A39-8E80-9C5EB7C88B44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{1EA2953D-6A80-4F35-A644-9DC50EFDF4AF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1EA2953D-6A80-4F35-A644-9DC50EFDF4AF}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="57">
   <si>
     <t>Traipú</t>
   </si>
@@ -147,9 +147,6 @@
   </si>
   <si>
     <t>Tobias Barreto</t>
-  </si>
-  <si>
-    <t>Tomar do Geru</t>
   </si>
   <si>
     <t>Anastácio</t>
@@ -646,31 +643,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84356141-46CF-43DA-9183-9D352FB20C42}">
-  <dimension ref="A1:D30"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D29"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="20.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="49.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="11.5546875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="20.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="49.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="3" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>8409</v>
       </c>
@@ -681,10 +678,10 @@
         <v>1</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>8140</v>
       </c>
@@ -695,10 +692,10 @@
         <v>3</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>8507</v>
       </c>
@@ -709,10 +706,10 @@
         <v>3</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>8102</v>
       </c>
@@ -723,10 +720,10 @@
         <v>3</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>8232</v>
       </c>
@@ -737,10 +734,10 @@
         <v>3</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>8581</v>
       </c>
@@ -751,10 +748,10 @@
         <v>8</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>8415</v>
       </c>
@@ -765,10 +762,10 @@
         <v>8</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>8354</v>
       </c>
@@ -779,10 +776,10 @@
         <v>8</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>8416</v>
       </c>
@@ -793,10 +790,10 @@
         <v>8</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>8340</v>
       </c>
@@ -807,10 +804,10 @@
         <v>8</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
         <v>8410</v>
       </c>
@@ -821,24 +818,24 @@
         <v>8</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
         <v>8683</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
         <v>8369</v>
       </c>
@@ -849,10 +846,10 @@
         <v>9</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
         <v>8090</v>
       </c>
@@ -863,10 +860,10 @@
         <v>7</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
         <v>8275</v>
       </c>
@@ -877,10 +874,10 @@
         <v>7</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
         <v>8582</v>
       </c>
@@ -891,10 +888,10 @@
         <v>7</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>8606</v>
       </c>
@@ -905,10 +902,10 @@
         <v>7</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
         <v>8149</v>
       </c>
@@ -919,10 +916,10 @@
         <v>7</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
         <v>8339</v>
       </c>
@@ -933,10 +930,10 @@
         <v>7</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
         <v>8118</v>
       </c>
@@ -947,10 +944,10 @@
         <v>7</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <v>8355</v>
       </c>
@@ -961,10 +958,10 @@
         <v>7</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
         <v>8326</v>
       </c>
@@ -975,10 +972,10 @@
         <v>4</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
         <v>8122</v>
       </c>
@@ -989,10 +986,10 @@
         <v>4</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
         <v>8314</v>
       </c>
@@ -1003,10 +1000,10 @@
         <v>6</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
         <v>8231</v>
       </c>
@@ -1017,10 +1014,10 @@
         <v>10</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
         <v>8091</v>
       </c>
@@ -1031,29 +1028,29 @@
         <v>10</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
-        <v>8279</v>
+        <v>8171</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>36</v>
+        <v>14</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="2">
-        <v>8171</v>
+        <v>8330</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>5</v>
@@ -1062,23 +1059,9 @@
         <v>49</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="2">
-        <v>8330</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>50</v>
-      </c>
-    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D30">
-    <sortCondition ref="C1:C30"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D29">
+    <sortCondition ref="C1:C29"/>
   </sortState>
   <conditionalFormatting sqref="A1:A1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>

</xml_diff>

<commit_message>
Atualiza nome_clientes.xlsx (26 -> 25 clientes)
Substitui pelo arquivo mais recente fornecido.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/nome_clientes.xlsx
+++ b/nome_clientes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FernandoHenriqueSofi\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96F437C8-4EFE-49DA-847F-AF6BB299A62A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6F8F756-EC0D-4A74-807A-A1273CDDD3EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-15" windowWidth="29040" windowHeight="16440" xr2:uid="{1EA2953D-6A80-4F35-A644-9DC50EFDF4AF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1EA2953D-6A80-4F35-A644-9DC50EFDF4AF}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="51">
   <si>
     <t>Carmo de Cachoeira</t>
   </si>
@@ -132,9 +132,6 @@
   </si>
   <si>
     <t>Lindóia</t>
-  </si>
-  <si>
-    <t>Nossa Senhora da Glória</t>
   </si>
   <si>
     <t>Tobias Barreto</t>
@@ -619,7 +616,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84356141-46CF-43DA-9183-9D352FB20C42}">
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.5546875" style="1" customWidth="1"/>
@@ -631,16 +628,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>36</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -654,7 +651,7 @@
         <v>5</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -668,7 +665,7 @@
         <v>4</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -682,7 +679,7 @@
         <v>1</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -696,7 +693,7 @@
         <v>1</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -710,7 +707,7 @@
         <v>7</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
@@ -724,7 +721,7 @@
         <v>6</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -732,13 +729,13 @@
         <v>8683</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -752,7 +749,7 @@
         <v>1</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -766,7 +763,7 @@
         <v>5</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -780,7 +777,7 @@
         <v>5</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
@@ -794,7 +791,7 @@
         <v>5</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
@@ -808,7 +805,7 @@
         <v>5</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -822,7 +819,7 @@
         <v>5</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
@@ -836,7 +833,7 @@
         <v>5</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
@@ -850,7 +847,7 @@
         <v>2</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
@@ -864,7 +861,7 @@
         <v>2</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
@@ -878,7 +875,7 @@
         <v>3</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
@@ -892,7 +889,7 @@
         <v>3</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
@@ -906,7 +903,7 @@
         <v>1</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
@@ -920,7 +917,7 @@
         <v>6</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
@@ -934,7 +931,7 @@
         <v>6</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
@@ -948,7 +945,7 @@
         <v>6</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
@@ -962,7 +959,7 @@
         <v>6</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
@@ -976,12 +973,12 @@
         <v>6</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
-        <v>8231</v>
+        <v>8091</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>31</v>
@@ -990,26 +987,12 @@
         <v>8</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" s="2">
-        <v>8091</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D27">
-    <sortCondition ref="D1:D27"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D26">
+    <sortCondition ref="D1:D26"/>
   </sortState>
   <conditionalFormatting sqref="A1:A1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>

</xml_diff>